<commit_message>
Order template: drop Needed vs Ordered sheet (purchase log only)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014FJcz4sTjvfWvU37rjR8pe
</commit_message>
<xml_diff>
--- a/tracker/templates/TEMPLATE_FiltersOrders.xlsx
+++ b/tracker/templates/TEMPLATE_FiltersOrders.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Needed vs Ordered" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Order Log'!$7:$7</definedName>
@@ -23,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,10 +41,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00595959"/>
     </font>
   </fonts>
   <fills count="4">
@@ -92,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -113,10 +108,6 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1784,582 +1775,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E42"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>NEEDED VS ORDERED</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>Type each size in Size. Count Needed and Still needed from the Filter Log. The other two columns fill in by themselves.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>Size</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>Ordered (all orders)</t>
-        </is>
-      </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>Needed - units replaced</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
-        <is>
-          <t>Left over (+) / Short (-)</t>
-        </is>
-      </c>
-      <c r="E3" s="10" t="inlineStr">
-        <is>
-          <t>Still needed - units not yet replaced</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6">
-        <f>IF(A4="","",SUMIF('Order Log'!$H$8:$H$67,A4,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6">
-        <f>IF(A4="","",B4-C4)</f>
-        <v/>
-      </c>
-      <c r="E4" s="6" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="6">
-        <f>IF(A5="","",SUMIF('Order Log'!$H$8:$H$67,A5,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6">
-        <f>IF(A5="","",B5-C5)</f>
-        <v/>
-      </c>
-      <c r="E5" s="6" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="n"/>
-      <c r="B6" s="6">
-        <f>IF(A6="","",SUMIF('Order Log'!$H$8:$H$67,A6,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6">
-        <f>IF(A6="","",B6-C6)</f>
-        <v/>
-      </c>
-      <c r="E6" s="6" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6">
-        <f>IF(A7="","",SUMIF('Order Log'!$H$8:$H$67,A7,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6">
-        <f>IF(A7="","",B7-C7)</f>
-        <v/>
-      </c>
-      <c r="E7" s="6" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6">
-        <f>IF(A8="","",SUMIF('Order Log'!$H$8:$H$67,A8,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6">
-        <f>IF(A8="","",B8-C8)</f>
-        <v/>
-      </c>
-      <c r="E8" s="6" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6">
-        <f>IF(A9="","",SUMIF('Order Log'!$H$8:$H$67,A9,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6">
-        <f>IF(A9="","",B9-C9)</f>
-        <v/>
-      </c>
-      <c r="E9" s="6" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n"/>
-      <c r="B10" s="6">
-        <f>IF(A10="","",SUMIF('Order Log'!$H$8:$H$67,A10,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6">
-        <f>IF(A10="","",B10-C10)</f>
-        <v/>
-      </c>
-      <c r="E10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n"/>
-      <c r="B11" s="6">
-        <f>IF(A11="","",SUMIF('Order Log'!$H$8:$H$67,A11,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6">
-        <f>IF(A11="","",B11-C11)</f>
-        <v/>
-      </c>
-      <c r="E11" s="6" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="n"/>
-      <c r="B12" s="6">
-        <f>IF(A12="","",SUMIF('Order Log'!$H$8:$H$67,A12,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6">
-        <f>IF(A12="","",B12-C12)</f>
-        <v/>
-      </c>
-      <c r="E12" s="6" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" s="6">
-        <f>IF(A13="","",SUMIF('Order Log'!$H$8:$H$67,A13,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6">
-        <f>IF(A13="","",B13-C13)</f>
-        <v/>
-      </c>
-      <c r="E13" s="6" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="n"/>
-      <c r="B14" s="6">
-        <f>IF(A14="","",SUMIF('Order Log'!$H$8:$H$67,A14,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6">
-        <f>IF(A14="","",B14-C14)</f>
-        <v/>
-      </c>
-      <c r="E14" s="6" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="6">
-        <f>IF(A15="","",SUMIF('Order Log'!$H$8:$H$67,A15,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6">
-        <f>IF(A15="","",B15-C15)</f>
-        <v/>
-      </c>
-      <c r="E15" s="6" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="n"/>
-      <c r="B16" s="6">
-        <f>IF(A16="","",SUMIF('Order Log'!$H$8:$H$67,A16,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6">
-        <f>IF(A16="","",B16-C16)</f>
-        <v/>
-      </c>
-      <c r="E16" s="6" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="6">
-        <f>IF(A17="","",SUMIF('Order Log'!$H$8:$H$67,A17,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6">
-        <f>IF(A17="","",B17-C17)</f>
-        <v/>
-      </c>
-      <c r="E17" s="6" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="n"/>
-      <c r="B18" s="6">
-        <f>IF(A18="","",SUMIF('Order Log'!$H$8:$H$67,A18,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6">
-        <f>IF(A18="","",B18-C18)</f>
-        <v/>
-      </c>
-      <c r="E18" s="6" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="6">
-        <f>IF(A19="","",SUMIF('Order Log'!$H$8:$H$67,A19,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6">
-        <f>IF(A19="","",B19-C19)</f>
-        <v/>
-      </c>
-      <c r="E19" s="6" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="6">
-        <f>IF(A20="","",SUMIF('Order Log'!$H$8:$H$67,A20,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6">
-        <f>IF(A20="","",B20-C20)</f>
-        <v/>
-      </c>
-      <c r="E20" s="6" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="6">
-        <f>IF(A21="","",SUMIF('Order Log'!$H$8:$H$67,A21,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6">
-        <f>IF(A21="","",B21-C21)</f>
-        <v/>
-      </c>
-      <c r="E21" s="6" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="n"/>
-      <c r="B22" s="6">
-        <f>IF(A22="","",SUMIF('Order Log'!$H$8:$H$67,A22,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C22" s="6" t="n"/>
-      <c r="D22" s="6">
-        <f>IF(A22="","",B22-C22)</f>
-        <v/>
-      </c>
-      <c r="E22" s="6" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6">
-        <f>IF(A23="","",SUMIF('Order Log'!$H$8:$H$67,A23,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6">
-        <f>IF(A23="","",B23-C23)</f>
-        <v/>
-      </c>
-      <c r="E23" s="6" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="n"/>
-      <c r="B24" s="6">
-        <f>IF(A24="","",SUMIF('Order Log'!$H$8:$H$67,A24,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C24" s="6" t="n"/>
-      <c r="D24" s="6">
-        <f>IF(A24="","",B24-C24)</f>
-        <v/>
-      </c>
-      <c r="E24" s="6" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="n"/>
-      <c r="B25" s="6">
-        <f>IF(A25="","",SUMIF('Order Log'!$H$8:$H$67,A25,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C25" s="6" t="n"/>
-      <c r="D25" s="6">
-        <f>IF(A25="","",B25-C25)</f>
-        <v/>
-      </c>
-      <c r="E25" s="6" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="n"/>
-      <c r="B26" s="6">
-        <f>IF(A26="","",SUMIF('Order Log'!$H$8:$H$67,A26,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6">
-        <f>IF(A26="","",B26-C26)</f>
-        <v/>
-      </c>
-      <c r="E26" s="6" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="n"/>
-      <c r="B27" s="6">
-        <f>IF(A27="","",SUMIF('Order Log'!$H$8:$H$67,A27,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C27" s="6" t="n"/>
-      <c r="D27" s="6">
-        <f>IF(A27="","",B27-C27)</f>
-        <v/>
-      </c>
-      <c r="E27" s="6" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="n"/>
-      <c r="B28" s="6">
-        <f>IF(A28="","",SUMIF('Order Log'!$H$8:$H$67,A28,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C28" s="6" t="n"/>
-      <c r="D28" s="6">
-        <f>IF(A28="","",B28-C28)</f>
-        <v/>
-      </c>
-      <c r="E28" s="6" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="n"/>
-      <c r="B29" s="6">
-        <f>IF(A29="","",SUMIF('Order Log'!$H$8:$H$67,A29,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C29" s="6" t="n"/>
-      <c r="D29" s="6">
-        <f>IF(A29="","",B29-C29)</f>
-        <v/>
-      </c>
-      <c r="E29" s="6" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="6">
-        <f>IF(A30="","",SUMIF('Order Log'!$H$8:$H$67,A30,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6">
-        <f>IF(A30="","",B30-C30)</f>
-        <v/>
-      </c>
-      <c r="E30" s="6" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="6" t="n"/>
-      <c r="B31" s="6">
-        <f>IF(A31="","",SUMIF('Order Log'!$H$8:$H$67,A31,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="6">
-        <f>IF(A31="","",B31-C31)</f>
-        <v/>
-      </c>
-      <c r="E31" s="6" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="n"/>
-      <c r="B32" s="6">
-        <f>IF(A32="","",SUMIF('Order Log'!$H$8:$H$67,A32,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="6">
-        <f>IF(A32="","",B32-C32)</f>
-        <v/>
-      </c>
-      <c r="E32" s="6" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="6">
-        <f>IF(A33="","",SUMIF('Order Log'!$H$8:$H$67,A33,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="6">
-        <f>IF(A33="","",B33-C33)</f>
-        <v/>
-      </c>
-      <c r="E33" s="6" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="n"/>
-      <c r="B34" s="6">
-        <f>IF(A34="","",SUMIF('Order Log'!$H$8:$H$67,A34,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C34" s="6" t="n"/>
-      <c r="D34" s="6">
-        <f>IF(A34="","",B34-C34)</f>
-        <v/>
-      </c>
-      <c r="E34" s="6" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="n"/>
-      <c r="B35" s="6">
-        <f>IF(A35="","",SUMIF('Order Log'!$H$8:$H$67,A35,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C35" s="6" t="n"/>
-      <c r="D35" s="6">
-        <f>IF(A35="","",B35-C35)</f>
-        <v/>
-      </c>
-      <c r="E35" s="6" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="n"/>
-      <c r="B36" s="6">
-        <f>IF(A36="","",SUMIF('Order Log'!$H$8:$H$67,A36,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C36" s="6" t="n"/>
-      <c r="D36" s="6">
-        <f>IF(A36="","",B36-C36)</f>
-        <v/>
-      </c>
-      <c r="E36" s="6" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="n"/>
-      <c r="B37" s="6">
-        <f>IF(A37="","",SUMIF('Order Log'!$H$8:$H$67,A37,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C37" s="6" t="n"/>
-      <c r="D37" s="6">
-        <f>IF(A37="","",B37-C37)</f>
-        <v/>
-      </c>
-      <c r="E37" s="6" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="n"/>
-      <c r="B38" s="6">
-        <f>IF(A38="","",SUMIF('Order Log'!$H$8:$H$67,A38,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C38" s="6" t="n"/>
-      <c r="D38" s="6">
-        <f>IF(A38="","",B38-C38)</f>
-        <v/>
-      </c>
-      <c r="E38" s="6" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="6" t="n"/>
-      <c r="B39" s="6">
-        <f>IF(A39="","",SUMIF('Order Log'!$H$8:$H$67,A39,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C39" s="6" t="n"/>
-      <c r="D39" s="6">
-        <f>IF(A39="","",B39-C39)</f>
-        <v/>
-      </c>
-      <c r="E39" s="6" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="n"/>
-      <c r="B40" s="6">
-        <f>IF(A40="","",SUMIF('Order Log'!$H$8:$H$67,A40,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C40" s="6" t="n"/>
-      <c r="D40" s="6">
-        <f>IF(A40="","",B40-C40)</f>
-        <v/>
-      </c>
-      <c r="E40" s="6" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="n"/>
-      <c r="B41" s="6">
-        <f>IF(A41="","",SUMIF('Order Log'!$H$8:$H$67,A41,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C41" s="6" t="n"/>
-      <c r="D41" s="6">
-        <f>IF(A41="","",B41-C41)</f>
-        <v/>
-      </c>
-      <c r="E41" s="6" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="n"/>
-      <c r="B42" s="6">
-        <f>IF(A42="","",SUMIF('Order Log'!$H$8:$H$67,A42,'Order Log'!$I$8:$I$67))</f>
-        <v/>
-      </c>
-      <c r="C42" s="6" t="n"/>
-      <c r="D42" s="6">
-        <f>IF(A42="","",B42-C42)</f>
-        <v/>
-      </c>
-      <c r="E42" s="6" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <conditionalFormatting sqref="A4:E42">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>MOD(ROW(),2)=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Order template: rename to Filter Orders
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014FJcz4sTjvfWvU37rjR8pe
</commit_message>
<xml_diff>
--- a/tracker/templates/TEMPLATE_FiltersOrders.xlsx
+++ b/tracker/templates/TEMPLATE_FiltersOrders.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Filter Orders" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Order Log'!$7:$7</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Filter Orders'!$7:$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -504,7 +504,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FILTER ORDER LOG</t>
+          <t>FILTER ORDERS</t>
         </is>
       </c>
     </row>

</xml_diff>